<commit_message>
chore(content): webp media migration, insights drafts, marketing content
- Remove superseded insights + Belmond PNGs (webp replacements in place;
  no code or DB references remain)
- Add web-optimized insights/demo imagery, blog drafts, HubSpot intro
  campaign, content blueprint, and insights seeding script

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/content-strategy/EAH_90_Day_Content_Calendar.xlsx
+++ b/marketing/content-strategy/EAH_90_Day_Content_Calendar.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1687,6 +1687,156 @@
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Thu Jul 16</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>The supplier catalog is the moat: what is built into every EAH site</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>travel advisor supplier catalog</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>BOFU</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Feature deep dive</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Real catalog numbers (~1,800 hotels, 20+ programs, 26 cruise lines). Extractable table = citable asset.</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Thu Jul 30</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>How the tiers stack: the modules that build a luxury advisor site</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>travel advisor website features</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>BOFU</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Feature walkthrough</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Stack-never-rebuild message. Respect tier gating. Tier table extractable.</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Thu Aug 13</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>How your journal stays alive without you writing every week</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>travel advisor blog content</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>BOFU</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>Feature post</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>Curated editorial stream (Growth+). Ties to dead-journal problem across cluster.</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>

</xml_diff>